<commit_message>
initital repo cleanup commit
</commit_message>
<xml_diff>
--- a/data/Labor Force Components.xlsx
+++ b/data/Labor Force Components.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sandag-my.sharepoint.com/personal/cra_sandag_org/Documents/Documents/GitHub/Population-Sim/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sandag-my.sharepoint.com/personal/gsc_sandag_org/Documents/VSCode Projects/Python/Population-Sim/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{50E35A42-41DA-4984-AC8F-0C8CF8CB411F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6FEED0E0-E717-42A6-8261-AEC0DAE8255A}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="8_{50E35A42-41DA-4984-AC8F-0C8CF8CB411F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{13319D60-8B28-4FD3-B3A8-BEC9F5F0C20C}"/>
   <bookViews>
-    <workbookView xWindow="23310" yWindow="2340" windowWidth="38700" windowHeight="15435" xr2:uid="{5B5C2CBC-A43D-4B4E-85EA-5E38A4C71155}"/>
+    <workbookView xWindow="14976" yWindow="0" windowWidth="14976" windowHeight="19368" xr2:uid="{5B5C2CBC-A43D-4B4E-85EA-5E38A4C71155}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -119,6 +119,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -439,13 +443,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A394A028-CB70-4417-BB56-679A465752C8}">
   <dimension ref="A1:N6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="1" max="1" width="10.5546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="32" customWidth="1"/>
-    <col min="4" max="14" width="9.140625" style="1"/>
+    <col min="3" max="3" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="14" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -480,7 +486,7 @@
         <v>2060</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -515,7 +521,7 @@
         <v>1593.8979170846201</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -550,7 +556,7 @@
         <v>619.38914994495201</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -585,7 +591,7 @@
         <v>54.768082607022102</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -620,7 +626,7 @@
         <v>391.22819840073203</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>3</v>
       </c>

</xml_diff>